<commit_message>
UPDATE: price format, liters format etc.
</commit_message>
<xml_diff>
--- a/SPLIT_COMPANY_DATA/RESULT/companies_result/ДОМАШЕН СОЦИАЛЕН ПАТРОНАЖ/ДОМАШЕН СОЦИАЛЕН ПАТРОНАЖ.xlsx
+++ b/SPLIT_COMPANY_DATA/RESULT/companies_result/ДОМАШЕН СОЦИАЛЕН ПАТРОНАЖ/ДОМАШЕН СОЦИАЛЕН ПАТРОНАЖ.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="69">
   <si>
     <t>Дата</t>
   </si>
@@ -34,6 +34,9 @@
     <t>Литри</t>
   </si>
   <si>
+    <t>Тип количество</t>
+  </si>
+  <si>
     <t>GTA цена</t>
   </si>
   <si>
@@ -55,115 +58,151 @@
     <t>Billing_Document</t>
   </si>
   <si>
-    <t>Варна Цар Освободител</t>
-  </si>
-  <si>
-    <t>Варна Варненчик</t>
-  </si>
-  <si>
-    <t>Варна Сливница</t>
-  </si>
-  <si>
-    <t>Варна Порт</t>
-  </si>
-  <si>
-    <t>Варна Евkсиноград</t>
+    <t>1147 Варна Ситроен</t>
+  </si>
+  <si>
+    <t>1911 O5 Варна</t>
+  </si>
+  <si>
+    <t>1148 Варна пристанище</t>
+  </si>
+  <si>
+    <t>1199 Varna Car Osvoboditel</t>
+  </si>
+  <si>
+    <t>B6386HH</t>
+  </si>
+  <si>
+    <t>B7846TP</t>
+  </si>
+  <si>
+    <t>B4160TK</t>
+  </si>
+  <si>
+    <t>B8917BP</t>
+  </si>
+  <si>
+    <t>B0452TC</t>
+  </si>
+  <si>
+    <t>B2207PP</t>
   </si>
   <si>
     <t>B4161TK</t>
   </si>
   <si>
-    <t>B5383XE</t>
-  </si>
-  <si>
-    <t>B7846TP</t>
-  </si>
-  <si>
-    <t>B8917BP</t>
-  </si>
-  <si>
-    <t>B6386HH</t>
-  </si>
-  <si>
-    <t>B4160TK</t>
+    <t>B5379XE</t>
   </si>
   <si>
     <t>B7845TP</t>
   </si>
   <si>
-    <t>B5379XE</t>
-  </si>
-  <si>
-    <t>B0452TC</t>
+    <t>78970155027721301</t>
+  </si>
+  <si>
+    <t>78970155027721194</t>
+  </si>
+  <si>
+    <t>78970155027721293</t>
+  </si>
+  <si>
+    <t>78970155027721269</t>
+  </si>
+  <si>
+    <t>78970155027721202</t>
+  </si>
+  <si>
+    <t>78970155027721178</t>
   </si>
   <si>
     <t>78970155027721285</t>
   </si>
   <si>
-    <t>78970155027721236</t>
-  </si>
-  <si>
-    <t>78970155027721194</t>
-  </si>
-  <si>
-    <t>78970155027721269</t>
-  </si>
-  <si>
-    <t>78970155027721301</t>
-  </si>
-  <si>
-    <t>78970155027721293</t>
+    <t>78970155027721244</t>
   </si>
   <si>
     <t>78970155027721251</t>
   </si>
   <si>
-    <t>78970155027721244</t>
-  </si>
-  <si>
-    <t>78970155027721202</t>
-  </si>
-  <si>
     <t>DIESEL EKONOMY</t>
   </si>
   <si>
-    <t>13:41</t>
-  </si>
-  <si>
-    <t>13:43</t>
-  </si>
-  <si>
-    <t>13:56</t>
-  </si>
-  <si>
-    <t>10:18</t>
-  </si>
-  <si>
-    <t>10:06</t>
-  </si>
-  <si>
-    <t>12:37</t>
-  </si>
-  <si>
-    <t>10:54</t>
-  </si>
-  <si>
-    <t>14:10</t>
-  </si>
-  <si>
-    <t>12:25</t>
-  </si>
-  <si>
-    <t>12:40</t>
-  </si>
-  <si>
-    <t>12:45</t>
-  </si>
-  <si>
-    <t>13:19</t>
-  </si>
-  <si>
-    <t>13:33</t>
+    <t>95 EKONOMY UNLEADED</t>
+  </si>
+  <si>
+    <t>L15</t>
+  </si>
+  <si>
+    <t>10:29:00</t>
+  </si>
+  <si>
+    <t>13:33:00</t>
+  </si>
+  <si>
+    <t>13:31:00</t>
+  </si>
+  <si>
+    <t>13:40:00</t>
+  </si>
+  <si>
+    <t>10:13:00</t>
+  </si>
+  <si>
+    <t>13:23:00</t>
+  </si>
+  <si>
+    <t>14:11:00</t>
+  </si>
+  <si>
+    <t>13:52:00</t>
+  </si>
+  <si>
+    <t>13:29:00</t>
+  </si>
+  <si>
+    <t>13:07:00</t>
+  </si>
+  <si>
+    <t>12:33:00</t>
+  </si>
+  <si>
+    <t>10:49:00</t>
+  </si>
+  <si>
+    <t>3236508147 3236508147</t>
+  </si>
+  <si>
+    <t>3236559755 3236559755</t>
+  </si>
+  <si>
+    <t>3236606812 3236606812</t>
+  </si>
+  <si>
+    <t>3236660105 3236660105</t>
+  </si>
+  <si>
+    <t>3236661468 3236661468</t>
+  </si>
+  <si>
+    <t>3236828268 3236828268</t>
+  </si>
+  <si>
+    <t>3236878929 3236878929</t>
+  </si>
+  <si>
+    <t>3236924571 3236924571</t>
+  </si>
+  <si>
+    <t>3236924950 3236924950</t>
+  </si>
+  <si>
+    <t>3236954992 3236954992</t>
+  </si>
+  <si>
+    <t>3237075098 3237075098</t>
+  </si>
+  <si>
+    <t>3237211433 3237211433</t>
   </si>
   <si>
     <t>Общи литри по продукт / ДОМАШЕН СОЦИАЛЕН ПАТРОНАЖ</t>
@@ -188,10 +227,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="#,##0.00"/>
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="#,##0.000"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-    <numFmt numFmtId="166" formatCode="#,##0.00000"/>
+    <numFmt numFmtId="166" formatCode="#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="#,##0.00000"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -271,7 +311,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -285,10 +325,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -583,7 +625,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M20"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="35.7109375" customWidth="1"/>
@@ -592,16 +634,17 @@
     <col min="4" max="4" width="28.7109375" customWidth="1"/>
     <col min="5" max="5" width="22.7109375" customWidth="1"/>
     <col min="6" max="6" width="18.7109375" customWidth="1"/>
-    <col min="7" max="7" width="15.7109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="16.7109375" customWidth="1"/>
     <col min="8" max="8" width="23.7109375" customWidth="1"/>
     <col min="9" max="9" width="15.7109375" style="1" customWidth="1"/>
     <col min="10" max="10" width="23.7109375" customWidth="1"/>
-    <col min="11" max="11" width="7.7109375" customWidth="1"/>
-    <col min="12" max="12" width="11.7109375" customWidth="1"/>
-    <col min="13" max="13" width="18.7109375" customWidth="1"/>
+    <col min="11" max="11" width="15.7109375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="10.7109375" customWidth="1"/>
+    <col min="13" max="13" width="11.7109375" customWidth="1"/>
+    <col min="14" max="14" width="23.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -641,13 +684,16 @@
       <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:13">
+      <c r="N1" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
       <c r="A2" s="3">
-        <v>46237</v>
+        <v>46251</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
         <v>18</v>
@@ -659,33 +705,36 @@
         <v>36</v>
       </c>
       <c r="F2">
-        <v>57</v>
-      </c>
-      <c r="G2" s="1">
-        <v>1.76</v>
-      </c>
-      <c r="H2">
-        <v>100.32</v>
+        <v>73.44</v>
+      </c>
+      <c r="G2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H2" s="1">
+        <v>1.657</v>
       </c>
       <c r="I2" s="1">
-        <v>1.79</v>
-      </c>
-      <c r="J2">
-        <v>102.03</v>
-      </c>
-      <c r="K2" t="s">
-        <v>37</v>
-      </c>
-      <c r="L2">
-        <v>55898</v>
+        <v>121.69</v>
+      </c>
+      <c r="J2" s="1">
+        <v>1.8</v>
+      </c>
+      <c r="K2" s="1">
+        <v>132.192</v>
+      </c>
+      <c r="L2" t="s">
+        <v>39</v>
       </c>
       <c r="M2">
-        <v>289167</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
+        <v>81063</v>
+      </c>
+      <c r="N2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" s="3">
-        <v>46237</v>
+        <v>46252</v>
       </c>
       <c r="B3" t="s">
         <v>14</v>
@@ -700,36 +749,39 @@
         <v>36</v>
       </c>
       <c r="F3">
-        <v>30</v>
-      </c>
-      <c r="G3" s="1">
-        <v>1.76</v>
-      </c>
-      <c r="H3">
-        <v>52.8</v>
+        <v>56.85</v>
+      </c>
+      <c r="G3" t="s">
+        <v>38</v>
+      </c>
+      <c r="H3" s="1">
+        <v>1.677</v>
       </c>
       <c r="I3" s="1">
-        <v>1.79</v>
-      </c>
-      <c r="J3">
-        <v>53.7</v>
-      </c>
-      <c r="K3" t="s">
-        <v>38</v>
-      </c>
-      <c r="L3">
-        <v>7520</v>
+        <v>95.337</v>
+      </c>
+      <c r="J3" s="1">
+        <v>1.8</v>
+      </c>
+      <c r="K3" s="1">
+        <v>102.33</v>
+      </c>
+      <c r="L3" t="s">
+        <v>40</v>
       </c>
       <c r="M3">
-        <v>134139</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
+        <v>32370</v>
+      </c>
+      <c r="N3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
       <c r="A4" s="3">
-        <v>46237</v>
+        <v>46253</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
         <v>20</v>
@@ -741,36 +793,39 @@
         <v>36</v>
       </c>
       <c r="F4">
-        <v>60.989</v>
-      </c>
-      <c r="G4" s="1">
-        <v>1.76</v>
-      </c>
-      <c r="H4">
-        <v>107.341</v>
+        <v>42.05</v>
+      </c>
+      <c r="G4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H4" s="1">
+        <v>1.677</v>
       </c>
       <c r="I4" s="1">
-        <v>1.79</v>
-      </c>
-      <c r="J4">
-        <v>109.17</v>
-      </c>
-      <c r="K4" t="s">
-        <v>39</v>
-      </c>
-      <c r="L4">
-        <v>32005</v>
+        <v>70.518</v>
+      </c>
+      <c r="J4" s="1">
+        <v>1.82</v>
+      </c>
+      <c r="K4" s="1">
+        <v>76.53100000000001</v>
+      </c>
+      <c r="L4" t="s">
+        <v>41</v>
       </c>
       <c r="M4">
-        <v>229284</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
+        <v>57925</v>
+      </c>
+      <c r="N4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
       <c r="A5" s="3">
-        <v>46238</v>
+        <v>46254</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
         <v>21</v>
@@ -784,31 +839,34 @@
       <c r="F5">
         <v>20</v>
       </c>
-      <c r="G5" s="1">
-        <v>1.77</v>
-      </c>
-      <c r="H5">
-        <v>35.4</v>
+      <c r="G5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H5" s="1">
+        <v>1.689</v>
       </c>
       <c r="I5" s="1">
-        <v>1.8</v>
-      </c>
-      <c r="J5">
-        <v>36</v>
-      </c>
-      <c r="K5" t="s">
-        <v>40</v>
-      </c>
-      <c r="L5">
-        <v>76600</v>
+        <v>33.78</v>
+      </c>
+      <c r="J5" s="1">
+        <v>1.84</v>
+      </c>
+      <c r="K5" s="1">
+        <v>36.8</v>
+      </c>
+      <c r="L5" t="s">
+        <v>42</v>
       </c>
       <c r="M5">
-        <v>158977</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
+        <v>76960</v>
+      </c>
+      <c r="N5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
       <c r="A6" s="3">
-        <v>46239</v>
+        <v>46254</v>
       </c>
       <c r="B6" t="s">
         <v>16</v>
@@ -823,36 +881,39 @@
         <v>36</v>
       </c>
       <c r="F6">
-        <v>61.378</v>
-      </c>
-      <c r="G6" s="1">
-        <v>1.77</v>
-      </c>
-      <c r="H6">
-        <v>108.639</v>
+        <v>50.01</v>
+      </c>
+      <c r="G6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H6" s="1">
+        <v>1.689</v>
       </c>
       <c r="I6" s="1">
-        <v>1.8</v>
-      </c>
-      <c r="J6">
-        <v>110.48</v>
-      </c>
-      <c r="K6" t="s">
-        <v>41</v>
-      </c>
-      <c r="L6">
-        <v>0</v>
+        <v>84.467</v>
+      </c>
+      <c r="J6" s="1">
+        <v>1.84</v>
+      </c>
+      <c r="K6" s="1">
+        <v>92.018</v>
+      </c>
+      <c r="L6" t="s">
+        <v>43</v>
       </c>
       <c r="M6">
-        <v>242427</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
+        <v>68230</v>
+      </c>
+      <c r="N6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
       <c r="A7" s="3">
-        <v>46239</v>
+        <v>46258</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C7" t="s">
         <v>23</v>
@@ -861,39 +922,42 @@
         <v>32</v>
       </c>
       <c r="E7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F7">
-        <v>38.761</v>
-      </c>
-      <c r="G7" s="1">
-        <v>1.77</v>
-      </c>
-      <c r="H7">
-        <v>68.607</v>
+        <v>50.66</v>
+      </c>
+      <c r="G7" t="s">
+        <v>38</v>
+      </c>
+      <c r="H7" s="1">
+        <v>1.439</v>
       </c>
       <c r="I7" s="1">
-        <v>1.8</v>
-      </c>
-      <c r="J7">
-        <v>69.77</v>
-      </c>
-      <c r="K7" t="s">
-        <v>42</v>
-      </c>
-      <c r="L7">
-        <v>57295</v>
+        <v>72.90000000000001</v>
+      </c>
+      <c r="J7" s="1">
+        <v>1.57</v>
+      </c>
+      <c r="K7" s="1">
+        <v>79.536</v>
+      </c>
+      <c r="L7" t="s">
+        <v>44</v>
       </c>
       <c r="M7">
-        <v>233343</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
+        <v>155190</v>
+      </c>
+      <c r="N7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
       <c r="A8" s="3">
-        <v>46244</v>
+        <v>46258</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C8" t="s">
         <v>24</v>
@@ -905,36 +969,39 @@
         <v>36</v>
       </c>
       <c r="F8">
-        <v>48</v>
-      </c>
-      <c r="G8" s="1">
-        <v>1.77</v>
-      </c>
-      <c r="H8">
-        <v>84.95999999999999</v>
+        <v>54.27</v>
+      </c>
+      <c r="G8" t="s">
+        <v>38</v>
+      </c>
+      <c r="H8" s="1">
+        <v>1.708</v>
       </c>
       <c r="I8" s="1">
-        <v>1.8</v>
-      </c>
-      <c r="J8">
-        <v>86.40000000000001</v>
-      </c>
-      <c r="K8" t="s">
-        <v>43</v>
-      </c>
-      <c r="L8">
-        <v>39185</v>
+        <v>92.693</v>
+      </c>
+      <c r="J8" s="1">
+        <v>1.85</v>
+      </c>
+      <c r="K8" s="1">
+        <v>100.4</v>
+      </c>
+      <c r="L8" t="s">
+        <v>45</v>
       </c>
       <c r="M8">
-        <v>161545</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
+        <v>56678</v>
+      </c>
+      <c r="N8" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
       <c r="A9" s="3">
-        <v>46244</v>
+        <v>46259</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C9" t="s">
         <v>25</v>
@@ -946,159 +1013,171 @@
         <v>36</v>
       </c>
       <c r="F9">
-        <v>73</v>
-      </c>
-      <c r="G9" s="1">
-        <v>1.77</v>
-      </c>
-      <c r="H9">
-        <v>129.21</v>
+        <v>50.02</v>
+      </c>
+      <c r="G9" t="s">
+        <v>38</v>
+      </c>
+      <c r="H9" s="1">
+        <v>1.719</v>
       </c>
       <c r="I9" s="1">
-        <v>1.8</v>
-      </c>
-      <c r="J9">
-        <v>131.4</v>
-      </c>
-      <c r="K9" t="s">
-        <v>44</v>
-      </c>
-      <c r="L9">
-        <v>7893</v>
+        <v>85.98399999999999</v>
+      </c>
+      <c r="J9" s="1">
+        <v>1.85</v>
+      </c>
+      <c r="K9" s="1">
+        <v>92.53700000000001</v>
+      </c>
+      <c r="L9" t="s">
+        <v>46</v>
       </c>
       <c r="M9">
-        <v>291410</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
+        <v>8430</v>
+      </c>
+      <c r="N9" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
       <c r="A10" s="3">
-        <v>46245</v>
+        <v>46259</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C10" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D10" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E10" t="s">
         <v>36</v>
       </c>
       <c r="F10">
-        <v>69.989</v>
-      </c>
-      <c r="G10" s="1">
-        <v>1.77</v>
-      </c>
-      <c r="H10">
-        <v>123.881</v>
+        <v>30</v>
+      </c>
+      <c r="G10" t="s">
+        <v>38</v>
+      </c>
+      <c r="H10" s="1">
+        <v>1.719</v>
       </c>
       <c r="I10" s="1">
-        <v>1.8</v>
-      </c>
-      <c r="J10">
-        <v>125.98</v>
-      </c>
-      <c r="K10" t="s">
-        <v>45</v>
-      </c>
-      <c r="L10">
-        <v>76558</v>
+        <v>51.57</v>
+      </c>
+      <c r="J10" s="1">
+        <v>1.85</v>
+      </c>
+      <c r="K10" s="1">
+        <v>55.5</v>
+      </c>
+      <c r="L10" t="s">
+        <v>47</v>
       </c>
       <c r="M10">
-        <v>291627</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13">
+        <v>39497</v>
+      </c>
+      <c r="N10" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
       <c r="A11" s="3">
-        <v>46246</v>
+        <v>46260</v>
       </c>
       <c r="B11" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C11" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D11" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E11" t="s">
         <v>36</v>
       </c>
       <c r="F11">
-        <v>41.889</v>
-      </c>
-      <c r="G11" s="1">
-        <v>1.77</v>
-      </c>
-      <c r="H11">
-        <v>74.14400000000001</v>
+        <v>38.44</v>
+      </c>
+      <c r="G11" t="s">
+        <v>38</v>
+      </c>
+      <c r="H11" s="1">
+        <v>1.719</v>
       </c>
       <c r="I11" s="1">
-        <v>1.8</v>
-      </c>
-      <c r="J11">
-        <v>75.40000000000001</v>
-      </c>
-      <c r="K11" t="s">
-        <v>46</v>
-      </c>
-      <c r="L11">
-        <v>57599</v>
+        <v>66.078</v>
+      </c>
+      <c r="J11" s="1">
+        <v>1.85</v>
+      </c>
+      <c r="K11" s="1">
+        <v>71.114</v>
+      </c>
+      <c r="L11" t="s">
+        <v>48</v>
       </c>
       <c r="M11">
-        <v>140061</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13">
+        <v>58220</v>
+      </c>
+      <c r="N11" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
       <c r="A12" s="3">
-        <v>46246</v>
+        <v>46262</v>
       </c>
       <c r="B12" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C12" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="D12" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E12" t="s">
         <v>36</v>
       </c>
       <c r="F12">
-        <v>35</v>
-      </c>
-      <c r="G12" s="1">
-        <v>1.77</v>
-      </c>
-      <c r="H12">
-        <v>61.95</v>
+        <v>68</v>
+      </c>
+      <c r="G12" t="s">
+        <v>38</v>
+      </c>
+      <c r="H12" s="1">
+        <v>1.719</v>
       </c>
       <c r="I12" s="1">
-        <v>1.8</v>
-      </c>
-      <c r="J12">
-        <v>63</v>
-      </c>
-      <c r="K12" t="s">
-        <v>47</v>
-      </c>
-      <c r="L12">
-        <v>67895</v>
+        <v>116.892</v>
+      </c>
+      <c r="J12" s="1">
+        <v>1.85</v>
+      </c>
+      <c r="K12" s="1">
+        <v>125.8</v>
+      </c>
+      <c r="L12" t="s">
+        <v>49</v>
       </c>
       <c r="M12">
-        <v>137725</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13">
+        <v>77403</v>
+      </c>
+      <c r="N12" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
       <c r="A13" s="3">
-        <v>46246</v>
+        <v>46265</v>
       </c>
       <c r="B13" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C13" t="s">
         <v>18</v>
@@ -1110,142 +1189,124 @@
         <v>36</v>
       </c>
       <c r="F13">
-        <v>48.25</v>
-      </c>
-      <c r="G13" s="1">
-        <v>1.77</v>
-      </c>
-      <c r="H13">
-        <v>85.402</v>
+        <v>40</v>
+      </c>
+      <c r="G13" t="s">
+        <v>38</v>
+      </c>
+      <c r="H13" s="1">
+        <v>1.719</v>
       </c>
       <c r="I13" s="1">
-        <v>1.8</v>
-      </c>
-      <c r="J13">
-        <v>86.84999999999999</v>
-      </c>
-      <c r="K13" t="s">
-        <v>48</v>
-      </c>
-      <c r="L13">
-        <v>79365</v>
+        <v>68.76000000000001</v>
+      </c>
+      <c r="J13" s="1">
+        <v>1.84</v>
+      </c>
+      <c r="K13" s="1">
+        <v>73.59999999999999</v>
+      </c>
+      <c r="L13" t="s">
+        <v>50</v>
       </c>
       <c r="M13">
-        <v>291898</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13">
-      <c r="A14" s="3">
-        <v>46246</v>
-      </c>
-      <c r="B14" t="s">
-        <v>14</v>
-      </c>
-      <c r="C14" t="s">
-        <v>19</v>
-      </c>
-      <c r="D14" t="s">
-        <v>28</v>
-      </c>
-      <c r="E14" t="s">
+        <v>81700</v>
+      </c>
+      <c r="N13" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14">
+      <c r="A16" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="F14">
-        <v>30</v>
-      </c>
-      <c r="G14" s="1">
-        <v>1.77</v>
-      </c>
-      <c r="H14">
-        <v>53.1</v>
-      </c>
-      <c r="I14" s="1">
-        <v>1.8</v>
-      </c>
-      <c r="J14">
-        <v>54</v>
-      </c>
-      <c r="K14" t="s">
-        <v>49</v>
-      </c>
-      <c r="L14">
-        <v>7805</v>
-      </c>
-      <c r="M14">
-        <v>137777</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6">
-      <c r="A17" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-    </row>
-    <row r="18" spans="1:6">
-      <c r="A18" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>9</v>
+      <c r="B18" s="7">
+        <v>523.08</v>
+      </c>
+      <c r="C18" s="8">
+        <v>11</v>
+      </c>
+      <c r="D18" s="9">
+        <v>1.6972</v>
+      </c>
+      <c r="E18" s="7">
+        <v>887.77</v>
+      </c>
+      <c r="F18" s="7">
+        <v>958.8200000000001</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B19" s="7">
-        <v>614.256</v>
-      </c>
-      <c r="C19" s="7">
-        <v>13</v>
-      </c>
-      <c r="D19" s="8">
-        <v>1.76759</v>
+        <v>50.66</v>
+      </c>
+      <c r="C19" s="8">
+        <v>1</v>
+      </c>
+      <c r="D19" s="9">
+        <v>1.43901</v>
       </c>
       <c r="E19" s="7">
-        <v>1085.75</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="F19" s="7">
-        <v>1104.18</v>
+        <v>79.54000000000001</v>
       </c>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="B20" s="10">
-        <v>614.256</v>
-      </c>
-      <c r="C20" s="10">
-        <v>13</v>
-      </c>
-      <c r="D20" s="8"/>
-      <c r="E20" s="10">
-        <v>1085.75</v>
-      </c>
-      <c r="F20" s="10">
-        <v>1104.18</v>
+      <c r="A20" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B20" s="11">
+        <v>573.74</v>
+      </c>
+      <c r="C20" s="12">
+        <v>12</v>
+      </c>
+      <c r="D20" s="9"/>
+      <c r="E20" s="11">
+        <v>960.67</v>
+      </c>
+      <c r="F20" s="11">
+        <v>1038.36</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A16:F16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>